<commit_message>
auto: snapshot 2026-07-28 13:31:00
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -4865,7 +4865,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-07-28 13:01:00</t>
+          <t>Timestamp: 2026-07-28 13:31:00</t>
         </is>
       </c>
     </row>
@@ -5283,11 +5283,11 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>24578</v>
+        <v>24662</v>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>+1008</t>
+          <t>+1092</t>
         </is>
       </c>
     </row>
@@ -5298,11 +5298,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>35318</v>
+        <v>35402</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+4161</t>
+          <t>+4245</t>
         </is>
       </c>
     </row>
@@ -5598,11 +5598,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>30856</v>
+        <v>30940</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+3805</t>
+          <t>+3889</t>
         </is>
       </c>
     </row>
@@ -5688,11 +5688,11 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>3333</v>
+        <v>3417</v>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>+3313</t>
+          <t>+3397</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-06 13:31:01
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -13664,7 +13664,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-06 13:01:00</t>
+          <t>Timestamp: 2026-08-06 13:31:00</t>
         </is>
       </c>
     </row>
@@ -14097,11 +14097,11 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>47746</v>
+        <v>47806</v>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>+672</t>
+          <t>+732</t>
         </is>
       </c>
     </row>
@@ -14337,11 +14337,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>16851</v>
+        <v>16911</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+1608</t>
+          <t>+1668</t>
         </is>
       </c>
     </row>
@@ -14397,11 +14397,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>59004</v>
+        <v>59054</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+3060</t>
+          <t>+3110</t>
         </is>
       </c>
     </row>
@@ -14457,11 +14457,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>32444</v>
+        <v>32504</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+2976</t>
+          <t>+3036</t>
         </is>
       </c>
     </row>
@@ -14487,11 +14487,11 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>18091</v>
+        <v>18151</v>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>+3012</t>
+          <t>+3072</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-07 13:01:01
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -30,6 +30,7 @@
     <sheet name="2026-08-04" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="2026-08-05" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="2026-08-06" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="2026-08-07" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -14519,6 +14520,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-07 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>300K Tokens LetsGo!</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>592</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>8310</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>320</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>621</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>250</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>9422</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>11960</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>9908</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+840</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>5589</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>32948</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>ZenithEX</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>48366</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>+560</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>8613</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>39762</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>350K All in</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>11534</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>3666</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>20222</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+3311</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Ary</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>300</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Morri§ey</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>24354</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>62816</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+3762</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>2060</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>35201</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+2697</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>900</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>21836</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+3685</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-08 13:01:01
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -31,6 +31,7 @@
     <sheet name="2026-08-05" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="2026-08-06" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="2026-08-07" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="2026-08-08" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -15399,6 +15400,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-08 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>961</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+961</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>300K Tokens LetsGo!</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>840</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>1389</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+797</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>9326</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>+1016</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>320</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>621</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>251</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Tuyu|Fortuners</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>+20</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>9422</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>11960</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>420</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+420</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>7282</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>10581</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>+673</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>5589</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>32948</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>BlacKoreana O</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>48823</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>8613</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>39762</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>350K All in</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>11534</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>2651</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>778</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>+778</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>57</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>3666</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>23025</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+2743</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>2400</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Ary</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>766</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>+466</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Morri§ey</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>25962</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+1608</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>65906</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+3030</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>1430</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>2070</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>1631</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>37509</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+2248</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>900</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>24752</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+2856</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-08 13:31:00
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -15424,7 +15424,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-08 13:01:00</t>
+          <t>Timestamp: 2026-08-08 13:31:00</t>
         </is>
       </c>
     </row>
@@ -16097,11 +16097,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>23025</v>
+        <v>23145</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+2743</t>
+          <t>+2863</t>
         </is>
       </c>
     </row>
@@ -16157,11 +16157,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>65906</v>
+        <v>66026</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+3030</t>
+          <t>+3150</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-10 13:01:01
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -33,6 +33,7 @@
     <sheet name="2026-08-07" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="2026-08-08" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="2026-08-09" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="2026-08-10" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17159,6 +17160,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-10 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>-29770</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>330</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>-25719</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>-21021</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>-23879</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>-29023</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>-19050</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>-16131</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>342</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>-39463</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>-15428</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>-18006</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>-29311</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>-21573</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>-25802</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>-28796</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>-28908</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>-37257</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>-36707</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>-14558</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>-27667</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>786</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>-26637</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>-28409</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>-35328</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>-39401</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>-27598</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>-28725</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>-59848</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>BlacKoreana O</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>-74851</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>-29535</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>-23520</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>683</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>-56271</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>-23635</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>-23619</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>-33785</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>-22392</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>-29661</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>-28816</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>-23421</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>-26957</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>-30793</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>-27113</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>-28524</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>-28683</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>-55017</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>-30999</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Ary</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>-29493</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Morri§ey</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>783</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>-46639</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>626</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>-95960</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>-29715</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>-30822</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>-23204</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>1257</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>-55536</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>-19547</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>1205</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>-52986</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>600</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>-27004</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-11 13:01:00
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -34,6 +34,7 @@
     <sheet name="2026-08-08" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="2026-08-09" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="2026-08-10" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="2026-08-11" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18039,6 +18040,885 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Shad0w Ninja Clan (105)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-08-11 13:01:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>dogan</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>NAOR</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>1393</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+1063</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Yata</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>AangEX</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Feirisu</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>£_Darkz_£</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>DangerousEX</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Xylota x [NvL]</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>3146</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>+2054</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>[R23] Wolf †</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Andrey</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>150</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>+150</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>MATHEMATRICK</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>BlacKAkiresu O</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>YE Brandy</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Khakashi Hatake</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ikhram </t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Kosaki</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Prince G™</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Yhwach Genryusai</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>NicolasRicko</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Izx Hatake Jr</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>3055</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>+2119</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>ASHBORN™</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Nabila|Fortuners</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>~[AnbuDream]~</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Ryujin Senju™</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heisenberg </t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Tobirama Senju™</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>BlacKoreana O</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>§åñÐåïmårµ | Frtners</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Meru™</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SNC | Vnzla Anbu |SN</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>683</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>SNC | Signature</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Fusion</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Sesshomaru</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>KYO</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitro </t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>SL41F3RT</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Flarekaze |Fortuners</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Raiden</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>ShadowRavenX</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Aldrin</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>SNC | TemperiTa</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>SmallDino</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Breaker LITE</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>1080</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>+1080</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Kokyotosu</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Ary</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Morri§ey</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>2306</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>+1523</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Jonny Brown</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>5335</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>+4409</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Knightwalker</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a fucking ninja </t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>+19</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Rood</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Aiah</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>2951</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>+1694</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>[R23] Cub †</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Izx Infernity </t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>5517</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>+4162</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>Erza Scarlet</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>600</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-11 13:31:00
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -18064,7 +18064,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-11 13:01:00</t>
+          <t>Timestamp: 2026-08-11 13:31:00</t>
         </is>
       </c>
     </row>
@@ -18782,11 +18782,11 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>2306</v>
+        <v>2391</v>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>+1523</t>
+          <t>+1608</t>
         </is>
       </c>
     </row>
@@ -18797,11 +18797,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>5335</v>
+        <v>5419</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+4409</t>
+          <t>+4493</t>
         </is>
       </c>
     </row>
@@ -18902,11 +18902,11 @@
         </is>
       </c>
       <c r="B58" s="5" t="n">
-        <v>600</v>
+        <v>698</v>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+98</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-12 13:31:00
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -18944,7 +18944,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-12 13:01:00</t>
+          <t>Timestamp: 2026-08-12 13:31:00</t>
         </is>
       </c>
     </row>
@@ -19617,11 +19617,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>4899</v>
+        <v>5007</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+3819</t>
+          <t>+3927</t>
         </is>
       </c>
     </row>
@@ -19677,11 +19677,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>10430</v>
+        <v>10538</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+5011</t>
+          <t>+5119</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-13 13:31:01
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -20703,7 +20703,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-13 13:01:00</t>
+          <t>Timestamp: 2026-08-13 13:31:00</t>
         </is>
       </c>
     </row>
@@ -20806,11 +20806,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>3452</v>
+        <v>3560</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+1944</t>
+          <t>+2052</t>
         </is>
       </c>
     </row>
@@ -21376,11 +21376,11 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>10032</v>
+        <v>10140</v>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>+5025</t>
+          <t>+5133</t>
         </is>
       </c>
     </row>
@@ -21436,11 +21436,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>14352</v>
+        <v>14478</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+3814</t>
+          <t>+3940</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-16 13:31:00
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -23343,7 +23343,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-16 13:01:00</t>
+          <t>Timestamp: 2026-08-16 13:31:00</t>
         </is>
       </c>
     </row>
@@ -24076,11 +24076,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>34554</v>
+        <v>34770</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+9942</t>
+          <t>+10158</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-20 13:31:01
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -26863,7 +26863,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-20 13:01:00</t>
+          <t>Timestamp: 2026-08-20 13:31:00</t>
         </is>
       </c>
     </row>
@@ -27596,11 +27596,11 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>59874</v>
+        <v>59982</v>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>+4668</t>
+          <t>+4776</t>
         </is>
       </c>
     </row>
@@ -27656,11 +27656,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>35655</v>
+        <v>35763</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+3786</t>
+          <t>+3894</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-08-29 13:31:02
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -35662,7 +35662,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-08-29 13:01:00</t>
+          <t>Timestamp: 2026-08-29 13:31:01</t>
         </is>
       </c>
     </row>
@@ -35765,11 +35765,11 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>8916</v>
+        <v>9036</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>+2820</t>
+          <t>+2940</t>
         </is>
       </c>
     </row>
@@ -35810,11 +35810,11 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>1782</v>
+        <v>1902</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>+1782</t>
+          <t>+1902</t>
         </is>
       </c>
     </row>
@@ -36050,11 +36050,11 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>2623</v>
+        <v>3223</v>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>+300</t>
+          <t>+900</t>
         </is>
       </c>
     </row>
@@ -36110,11 +36110,11 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>22852</v>
+        <v>22972</v>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>+1320</t>
+          <t>+1440</t>
         </is>
       </c>
     </row>
@@ -36155,11 +36155,11 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>49892</v>
+        <v>50012</v>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>+2040</t>
+          <t>+2160</t>
         </is>
       </c>
     </row>
@@ -36185,11 +36185,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>7420</v>
+        <v>7540</v>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>+2802</t>
+          <t>+2922</t>
         </is>
       </c>
     </row>
@@ -36410,11 +36410,11 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>104282</v>
+        <v>104402</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>+2894</t>
+          <t>+3014</t>
         </is>
       </c>
     </row>
@@ -36485,11 +36485,11 @@
         </is>
       </c>
       <c r="B57" s="5" t="n">
-        <v>46946</v>
+        <v>47066</v>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>+2812</t>
+          <t>+2932</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-12 13:31:01
</commit_message>
<xml_diff>
--- a/clan_105.xlsx
+++ b/clan_105.xlsx
@@ -49740,7 +49740,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-12 13:01:00</t>
+          <t>Timestamp: 2026-09-12 13:31:00</t>
         </is>
       </c>
     </row>
@@ -50488,11 +50488,11 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>37965</v>
+        <v>38085</v>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>+2330</t>
+          <t>+2450</t>
         </is>
       </c>
     </row>
@@ -50533,11 +50533,11 @@
         </is>
       </c>
       <c r="B55" s="5" t="n">
-        <v>31584</v>
+        <v>31685</v>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>+2631</t>
+          <t>+2732</t>
         </is>
       </c>
     </row>

</xml_diff>